<commit_message>
thong ke BBGN theplong
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/PKH_HRC1_BBGN_ThepLong.xlsx
+++ b/dataproduct.api/wwwroot/templates/PKH_HRC1_BBGN_ThepLong.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3ECB613-E357-41AD-BA35-61DD5FA5D94B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38148D32-C43F-4C61-8694-D115C63BF7E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>STT</t>
   </si>
@@ -40,9 +40,6 @@
     <t>Mác thép</t>
   </si>
   <si>
-    <t>Nhóm phân loại</t>
-  </si>
-  <si>
     <t>Thùng số</t>
   </si>
   <si>
@@ -79,10 +76,31 @@
     <t>Thử nghiệm</t>
   </si>
   <si>
-    <t>KL 1 cẩu</t>
-  </si>
-  <si>
-    <t>KL 2 cẩu</t>
+    <t>Kíp</t>
+  </si>
+  <si>
+    <t>Tình trạng lò thổi</t>
+  </si>
+  <si>
+    <t>Ngày Nhận Tinh Luyện</t>
+  </si>
+  <si>
+    <t>Tình trạng Tinh Luyện</t>
+  </si>
+  <si>
+    <t>Trạng thái chốt</t>
+  </si>
+  <si>
+    <t>Họ tên người sửa cuối lò thổi</t>
+  </si>
+  <si>
+    <t>Họ tên người sửa cuối Tinh luyện</t>
+  </si>
+  <si>
+    <t>Trạng thái xác nhận</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Họ tên người xác nhận cuối </t>
   </si>
 </sst>
 </file>
@@ -143,10 +161,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -478,94 +496,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:V4"/>
+  <dimension ref="A3:AA4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
     <col min="8" max="8" width="12.140625" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" customWidth="1"/>
     <col min="10" max="10" width="16.42578125" customWidth="1"/>
     <col min="11" max="11" width="14.5703125" customWidth="1"/>
     <col min="12" max="12" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" customWidth="1"/>
-    <col min="15" max="15" width="13.140625" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" customWidth="1"/>
-    <col min="18" max="18" width="16.42578125" customWidth="1"/>
+    <col min="13" max="14" width="11.42578125" customWidth="1"/>
+    <col min="15" max="16" width="13.28515625" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" customWidth="1"/>
+    <col min="18" max="18" width="17.140625" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" customWidth="1"/>
+    <col min="20" max="21" width="16.42578125" customWidth="1"/>
+    <col min="22" max="22" width="14.140625" customWidth="1"/>
+    <col min="23" max="23" width="18.7109375" customWidth="1"/>
+    <col min="24" max="26" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:22" ht="45.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="3" spans="1:27" ht="45.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P4" s="2" t="s">
+      <c r="R4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="S4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" s="2" t="s">
+      <c r="U4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V4" s="1"/>
+      <c r="W4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>